<commit_message>
refactor: import excel — cluster/harga/tgl tagih per baris, template di modal
- Kolom template: NAMA, WA, PAKET, HARGA, CLUSTER, ALAMAT, TGL TAGIH, KET., MAPS
- Cluster resolve by name per baris (opsional, assign via UI bila kosong) — cluster_id nullable
- Tombol Download Template pindah ke dalam modal import
- HARGA prioritas di atas harga paket; TGL TAGIH → billing_day (invalid → 1)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_pelanggan.xlsx
+++ b/tests/fixtures/sample_pelanggan.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="49">
   <si>
     <t>NAMA</t>
   </si>
@@ -26,9 +26,18 @@
     <t>PAKET</t>
   </si>
   <si>
+    <t>HARGA</t>
+  </si>
+  <si>
+    <t>CLUSTER</t>
+  </si>
+  <si>
     <t>ALAMAT</t>
   </si>
   <si>
+    <t>TGL TAGIH</t>
+  </si>
+  <si>
     <t>KET.</t>
   </si>
   <si>
@@ -38,6 +47,9 @@
     <t>Budi</t>
   </si>
   <si>
+    <t>PADI</t>
+  </si>
+  <si>
     <t>PADI 1</t>
   </si>
   <si>
@@ -59,6 +71,9 @@
     <t>Joko</t>
   </si>
   <si>
+    <t>padi</t>
+  </si>
+  <si>
     <t>PADI 3</t>
   </si>
   <si>
@@ -74,6 +89,9 @@
     <t>081234567803</t>
   </si>
   <si>
+    <t>KAPAS</t>
+  </si>
+  <si>
     <t>KAPAS 1</t>
   </si>
   <si>
@@ -95,6 +113,9 @@
     <t>Wati</t>
   </si>
   <si>
+    <t>JATI</t>
+  </si>
+  <si>
     <t>KAPAS 3</t>
   </si>
   <si>
@@ -132,6 +153,9 @@
   </si>
   <si>
     <t>081234567809</t>
+  </si>
+  <si>
+    <t>kapas</t>
   </si>
   <si>
     <t>JATI 4</t>
@@ -477,10 +501,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -499,10 +523,19 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>6282260000000.0</v>
@@ -510,36 +543,51 @@
       <c r="C2">
         <v>110</v>
       </c>
-      <c r="D2" t="s">
-        <v>7</v>
+      <c r="D2">
+        <v>110000</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>110</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3">
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>6281234567802</v>
@@ -547,133 +595,181 @@
       <c r="C4">
         <v>100</v>
       </c>
-      <c r="D4" t="s">
-        <v>14</v>
+      <c r="D4">
+        <v>100</v>
       </c>
       <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4">
         <v>15</v>
       </c>
-      <c r="F4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C5">
         <v>110</v>
       </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
       <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C6">
         <v>115</v>
       </c>
-      <c r="D6" t="s">
-        <v>23</v>
-      </c>
       <c r="E6" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>29</v>
+      </c>
+      <c r="G6">
+        <v>25</v>
+      </c>
+      <c r="H6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C7">
         <v>110</v>
       </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
       <c r="E7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>32</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>110</v>
       </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C9">
         <v>110</v>
       </c>
-      <c r="D9" t="s">
-        <v>33</v>
+      <c r="D9">
+        <v>120000</v>
       </c>
       <c r="E9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>24</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9">
+        <v>10</v>
+      </c>
+      <c r="H9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C10">
         <v>999</v>
       </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
       <c r="E10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C11">
         <v>110</v>
       </c>
-      <c r="D11" t="s">
-        <v>39</v>
-      </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>46</v>
+      </c>
+      <c r="F11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11">
+        <v>28</v>
+      </c>
+      <c r="H11" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>